<commit_message>
OS reset - 23/10/2026
</commit_message>
<xml_diff>
--- a/SEM 7/Progress.xlsx
+++ b/SEM 7/Progress.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\degree\SEM 7\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0905CD51-CE83-4C16-BBE1-6C66C5142547}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F147BA9-272F-41DA-9741-1DC16F7AD35C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="24">
   <si>
     <t>EXP1</t>
   </si>
@@ -100,16 +100,13 @@
   </si>
   <si>
     <t>Mini Project</t>
-  </si>
-  <si>
-    <t>Incomplete</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -161,21 +158,8 @@
       <name val="Microsoft JhengHei"/>
       <family val="2"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Microsoft JhengHei"/>
-      <family val="2"/>
-    </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -192,11 +176,6 @@
         <fgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -207,13 +186,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="4">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -226,13 +204,9 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="4">
+  <cellStyles count="3">
     <cellStyle name="Accent3" xfId="1" builtinId="37"/>
-    <cellStyle name="Bad" xfId="3" builtinId="27"/>
     <cellStyle name="Good" xfId="2" builtinId="26"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
@@ -820,8 +794,8 @@
       <c r="C21" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="D21" s="6" t="s">
-        <v>24</v>
+      <c r="D21" s="5" t="s">
+        <v>22</v>
       </c>
       <c r="E21" s="5" t="s">
         <v>22</v>
@@ -840,8 +814,8 @@
       <c r="C23" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="D23" s="6" t="s">
-        <v>24</v>
+      <c r="D23" s="5" t="s">
+        <v>22</v>
       </c>
       <c r="E23" s="4" t="s">
         <v>15</v>

</xml_diff>